<commit_message>
Export Language KO again and fill EN column
KO is per-language output text, so it is exported (the only Korean
exception). EN: proper nouns romanized, skills and UI translated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CDH3mwZmVtgx1ALhFj2DHN
</commit_message>
<xml_diff>
--- a/tables/Language.xlsx
+++ b/tables/Language.xlsx
@@ -457,7 +457,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>한 행 = 화면에 보이는 문구 하나. 다른 시트는 TextID(이 ID)로만 가리킨다. KO는 기획용 참고(비고 열, 추출에서 빠짐, 한국어 표시는 개발에서 하드코딩, 10/29). EN은 예비.</t>
+          <t>한 행 = 화면에 보이는 문구 하나. 다른 시트는 TextID(이 ID)로만 가리킨다. KO·EN은 언어별 출력 문구라 추출함(KO 한글은 이 시트만 예외, 10/29 개발팀 확인). EN 표기: 인물·요괴·보스·무기·지명 같은 고유명사는 로마자(국어의 로마자 표기법, 예: 막손 Makson), 수식어는 번역(불붙은 허수귀 Burning Heosugwi), 스킬·UI 문구는 영어 번역.</t>
         </is>
       </c>
       <c r="C1" s="1" t="n"/>
@@ -471,7 +471,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>CSV,표시 텍스트 ID(한글 문구는 추출하지 않음).</t>
+          <t>CSV,표시 텍스트 ID·언어별 문구(KO·EN).</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -513,7 +513,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>Name, KO, Note</t>
+          <t>Name, Note</t>
         </is>
       </c>
       <c r="C5" s="1" t="n"/>
@@ -560,6 +560,11 @@
           <t>막손</t>
         </is>
       </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Makson</t>
+        </is>
+      </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
           <t>주인공</t>
@@ -580,6 +585,11 @@
           <t>허수귀</t>
         </is>
       </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Heosugwi</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -595,6 +605,11 @@
           <t>지게귀</t>
         </is>
       </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Jigegwi</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -610,6 +625,11 @@
           <t>불붙은 허수귀</t>
         </is>
       </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Burning Heosugwi</t>
+        </is>
+      </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
           <t>변종</t>
@@ -630,6 +650,11 @@
           <t>짐 던지는 지게귀</t>
         </is>
       </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Pack-Throwing Jigegwi</t>
+        </is>
+      </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
           <t>변종</t>
@@ -650,6 +675,11 @@
           <t>쇄문아비</t>
         </is>
       </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Swaemunabi</t>
+        </is>
+      </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
           <t>보스</t>
@@ -670,6 +700,11 @@
           <t>발골칼</t>
         </is>
       </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Balgolkal</t>
+        </is>
+      </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
           <t>아이템 아님(해체 연출용). 지금 참조하는 행 없음</t>
@@ -690,6 +725,11 @@
           <t>버선칼</t>
         </is>
       </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Beoseonkal</t>
+        </is>
+      </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
           <t>시작 무기</t>
@@ -710,6 +750,11 @@
           <t>쇠메</t>
         </is>
       </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Soeme</t>
+        </is>
+      </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
           <t>완성판</t>
@@ -730,6 +775,11 @@
           <t>결박 가르기</t>
         </is>
       </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Bind Cleave</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -745,6 +795,11 @@
           <t>도화골</t>
         </is>
       </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Dohwagol</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -760,6 +815,11 @@
           <t>사냥터 1</t>
         </is>
       </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Hunting Ground 1</t>
+        </is>
+      </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
           <t>이름 미정</t>
@@ -780,6 +840,11 @@
           <t>사냥터 2</t>
         </is>
       </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Hunting Ground 2</t>
+        </is>
+      </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
           <t>이름 미정</t>
@@ -800,6 +865,11 @@
           <t>보스방</t>
         </is>
       </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Boss Room</t>
+        </is>
+      </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
           <t>이름 미정</t>
@@ -820,6 +890,11 @@
           <t>베기</t>
         </is>
       </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Slash</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -835,6 +910,11 @@
           <t>베기</t>
         </is>
       </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Slash</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -850,6 +930,11 @@
           <t>내리베기</t>
         </is>
       </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Downward Slash</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -865,6 +950,11 @@
           <t>공중 베기</t>
         </is>
       </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Aerial Slash</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -880,6 +970,11 @@
           <t>해체</t>
         </is>
       </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Carve</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -895,6 +990,11 @@
           <t>결박 가르기</t>
         </is>
       </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Bind Cleave</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -910,6 +1010,11 @@
           <t>회피</t>
         </is>
       </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Dodge</t>
+        </is>
+      </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
           <t>회피 확률 발동 시 표시</t>
@@ -930,6 +1035,11 @@
           <t>약초</t>
         </is>
       </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Herb</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -945,6 +1055,11 @@
           <t>결박 가르기를 익혔다</t>
         </is>
       </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Learned Bind Cleave</t>
+        </is>
+      </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
           <t>장부방</t>
@@ -965,6 +1080,11 @@
           <t>기록했다</t>
         </is>
       </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Progress recorded</t>
+        </is>
+      </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
           <t>저장 지점</t>
@@ -985,6 +1105,11 @@
           <t>TO BE CONTINUED</t>
         </is>
       </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>TO BE CONTINUED</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -998,6 +1123,11 @@
       <c r="C32" s="3" t="inlineStr">
         <is>
           <t>불러오는 중</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Language 30011~30014 맵 이름을 10/29 확정 이름으로
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CDH3mwZmVtgx1ALhFj2DHN
</commit_message>
<xml_diff>
--- a/tables/Language.xlsx
+++ b/tables/Language.xlsx
@@ -787,7 +787,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>마을 이름</t>
+          <t>맵 1 이름</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -807,22 +807,22 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>사냥터 1 이름</t>
+          <t>맵 2 이름</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>사냥터 1</t>
+          <t>산길 초입구</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Hunting Ground 1</t>
+          <t>Mountain Trail Entrance</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>이름 미정</t>
+          <t>10/29 확정</t>
         </is>
       </c>
     </row>
@@ -832,22 +832,22 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>사냥터 2 이름</t>
+          <t>맵 3 이름</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>사냥터 2</t>
+          <t>산길 위 바위 협곡</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Hunting Ground 2</t>
+          <t>Rocky Gorge Above the Trail</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>이름 미정</t>
+          <t>10/29 확정</t>
         </is>
       </c>
     </row>
@@ -857,22 +857,22 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>보스방 이름</t>
+          <t>맵 4 이름(보스)</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>보스방</t>
+          <t>관문</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Boss Room</t>
+          <t>The Gate</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>이름 미정</t>
+          <t>10/29 확정</t>
         </is>
       </c>
     </row>

</xml_diff>